<commit_message>
data: import feedbacks formation F-2026-003 à F-2026-008 (42 retours)
</commit_message>
<xml_diff>
--- a/public/data/suivi_presence_consultants.xlsx
+++ b/public/data/suivi_presence_consultants.xlsx
@@ -4014,256 +4014,1630 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="32">
-      <c r="C9" s="62" t="n"/>
-      <c r="F9" s="36" t="n"/>
-      <c r="G9" s="36" t="n"/>
-      <c r="H9" s="36" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>r-006</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>F-2026-003</t>
+        </is>
+      </c>
+      <c r="C9" s="63" t="n">
+        <v>46064.64322916666</v>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F9" s="36" t="inlineStr">
+        <is>
+          <t>Use case débrouillardise illustrant bien et retour d’expérience PM</t>
+        </is>
+      </c>
+      <c r="G9" s="36" t="inlineStr">
+        <is>
+          <t>Pas d’avis</t>
+        </is>
+      </c>
+      <c r="H9" s="36" t="inlineStr">
+        <is>
+          <t>Merci!!!</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="32">
-      <c r="C10" s="62" t="n"/>
-      <c r="F10" s="36" t="n"/>
-      <c r="G10" s="36" t="n"/>
-      <c r="H10" s="36" t="n"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>r-007</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>F-2026-003</t>
+        </is>
+      </c>
+      <c r="C10" s="63" t="n">
+        <v>46064.64791666667</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F10" s="36" t="inlineStr">
+        <is>
+          <t>les uses cases</t>
+        </is>
+      </c>
+      <c r="G10" s="36" t="inlineStr">
+        <is>
+          <t>Le deuxième use case est perfectible</t>
+        </is>
+      </c>
+      <c r="H10" s="36" t="inlineStr"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="32">
-      <c r="C11" s="62" t="n"/>
-      <c r="F11" s="36" t="n"/>
-      <c r="G11" s="36" t="n"/>
-      <c r="H11" s="36" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>r-008</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>F-2026-003</t>
+        </is>
+      </c>
+      <c r="C11" s="63" t="n">
+        <v>46064.65319444444</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Oui mais j'ai besoin de plus de pratique</t>
+        </is>
+      </c>
+      <c r="F11" s="36" t="inlineStr">
+        <is>
+          <t>La sympathie du coach</t>
+        </is>
+      </c>
+      <c r="G11" s="36" t="inlineStr">
+        <is>
+          <t>Recommandations :
+- Après la théorie, consacrer 10-15 min à la compréhension de Postman (fonctionnement de l'interface, possibilités d'interaction, etc.).
+- Présenter 2-3 use cases déjà résolus pour illustrer des scénarios concrets
+- Pendant le cas pratique, laisser 5min par question aux participants pour répondre, puis présenter le corrigé
+- Proposer d'autres exercices à faire plus tard en autonomie
+- Lister des ressources utiles pour continuer d'apprendre (autres use cases par exemple)</t>
+        </is>
+      </c>
+      <c r="H11" s="36" t="inlineStr">
+        <is>
+          <t>Merci pour cet atelier :)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="32">
-      <c r="C12" s="62" t="n"/>
-      <c r="F12" s="36" t="n"/>
-      <c r="G12" s="36" t="n"/>
-      <c r="H12" s="36" t="n"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>r-009</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>F-2026-003</t>
+        </is>
+      </c>
+      <c r="C12" s="63" t="n">
+        <v>46064.66564814815</v>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F12" s="36" t="inlineStr">
+        <is>
+          <t>J'ai particulièrement apprécié le format très orienté pratique, avec une part accordée aux exercices sur Postman beaucoup plus importante que ce que l'on voit d'habitude.
+Le choix de passer rapidement sur la théorie était très pertinent aussi. En tant que PO nous avons souvent déjà quelques bases, et cela nous a évité de perdre du temps sur des concepts déjà connus.</t>
+        </is>
+      </c>
+      <c r="G12" s="36" t="inlineStr">
+        <is>
+          <t>Pour moi il faut changer le cas pratique, la doc de PokeAPI est vraiment éclatée au sol, c'est pas l'idéal pour une premiere approche. Penser aussi à donner quelques indices ou pistes pendant les exercices pour éviter que certains restent bloqués sur les premières questions et ratent la suite.
+Personnellement ce qui m'a perturbé est une chose assez basique. Dans la première question du cas pratique. On doit ajouter un "/limit=151" dans le endpoint, alors que nous n'avons pas du tout parlé de cela dans la présentation, du coup si on ne sait pas comment ca fonctionne on peut chercher tres longtemps... c'est dommage car au final est hyper simple.
++ Je pense que ca serait intéressant dans la partie théorie de la pres de parler de la structure d'une API (params/header/body/test etc)</t>
+        </is>
+      </c>
+      <c r="H12" s="36" t="inlineStr">
+        <is>
+          <t>Pour moi la mise en pratique est essentielle surtout sur des sujets techniques comme celui-ci. Je pense que c’est le meilleur moyen de comprendre et de retenir. Une approche efficace que je recommande de généraliser !
+Je trouve cela très bénéfique pour nous de suivre des formations plus techniques (infrastructure, code, architecture...)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="32">
-      <c r="C13" s="62" t="n"/>
-      <c r="F13" s="36" t="n"/>
-      <c r="G13" s="36" t="n"/>
-      <c r="H13" s="36" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>r-010</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>F-2026-003</t>
+        </is>
+      </c>
+      <c r="C13" s="63" t="n">
+        <v>46064.81310185185</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Oui mais j'ai besoin de plus de pratique</t>
+        </is>
+      </c>
+      <c r="F13" s="36" t="inlineStr">
+        <is>
+          <t>les exercices a la fin</t>
+        </is>
+      </c>
+      <c r="G13" s="36" t="inlineStr">
+        <is>
+          <t>la correction des exercices en séance</t>
+        </is>
+      </c>
+      <c r="H13" s="36" t="inlineStr">
+        <is>
+          <t>merci !</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="32">
-      <c r="C14" s="62" t="n"/>
-      <c r="F14" s="36" t="n"/>
-      <c r="G14" s="36" t="n"/>
-      <c r="H14" s="36" t="n"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>r-011</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>F-2026-003</t>
+        </is>
+      </c>
+      <c r="C14" s="63" t="n">
+        <v>46065</v>
+      </c>
+      <c r="D14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Oui mais j'ai besoin de plus de pratique</t>
+        </is>
+      </c>
+      <c r="F14" s="36" t="inlineStr">
+        <is>
+          <t>La partie pratique</t>
+        </is>
+      </c>
+      <c r="G14" s="36" t="inlineStr">
+        <is>
+          <t>Dans la partie pratique, j'aurais bien aimé avoir plus d'explications de la part de Simon sur la méthodologie et une démo de comment il aurait fait après chaque étape.</t>
+        </is>
+      </c>
+      <c r="H14" s="36" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="32">
-      <c r="C15" s="62" t="n"/>
-      <c r="F15" s="36" t="n"/>
-      <c r="G15" s="36" t="n"/>
-      <c r="H15" s="36" t="n"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>r-012</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>F-2026-003</t>
+        </is>
+      </c>
+      <c r="C15" s="63" t="n">
+        <v>46065.37700231482</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F15" s="36" t="inlineStr">
+        <is>
+          <t>La mise en pratique avec Postman :)</t>
+        </is>
+      </c>
+      <c r="G15" s="36" t="inlineStr">
+        <is>
+          <t>Un peu plus de temps sur le théorique selon le niveau de l'assistance :)</t>
+        </is>
+      </c>
+      <c r="H15" s="36" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="32">
-      <c r="C16" s="62" t="n"/>
-      <c r="F16" s="36" t="n"/>
-      <c r="G16" s="36" t="n"/>
-      <c r="H16" s="36" t="n"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>r-013</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>F-2026-003</t>
+        </is>
+      </c>
+      <c r="C16" s="63" t="n">
+        <v>46065.68857638889</v>
+      </c>
+      <c r="D16" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Oui mais j'ai besoin de plus de pratique</t>
+        </is>
+      </c>
+      <c r="F16" s="36" t="inlineStr">
+        <is>
+          <t>Pratique</t>
+        </is>
+      </c>
+      <c r="G16" s="36" t="inlineStr">
+        <is>
+          <t>Plus de schémas logiques pour aider à la compréhension 
+Plus de cas d’usage mission pour un PM</t>
+        </is>
+      </c>
+      <c r="H16" s="36" t="inlineStr">
+        <is>
+          <t>Merci l’équipe formation 🫶🏻</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="32">
-      <c r="C17" s="62" t="n"/>
-      <c r="F17" s="36" t="n"/>
-      <c r="G17" s="36" t="n"/>
-      <c r="H17" s="36" t="n"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>r-014</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>F-2026-004</t>
+        </is>
+      </c>
+      <c r="C17" s="63" t="n">
+        <v>46078.4725925926</v>
+      </c>
+      <c r="D17" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F17" s="36" t="inlineStr">
+        <is>
+          <t>La partie théorique était top et super rythmée (alors que c’est souvent le plus « long » pour ceux qui écoutent) moi c’est la partie que j’ai préféré pour une fois avec notamment le retour de Antho qui était super intéressant !!</t>
+        </is>
+      </c>
+      <c r="G17" s="36" t="inlineStr">
+        <is>
+          <t>La partie pratique par contre j’ai été un peu frustrée par le « peu » de temps qu’on a eue et surtout que c’était très très guidé fin on s’est pas posé beaucoup de questions : je sais pas si c’est suffisant pour que quelqu’un derrière réussisse à en refaire un tout seul en autonomie…
+Mais je sais pas comment encourager les gens à le faire ! Peut être un concours de l’agent le plus wtf ??
+Ou un canal dédié IA ?</t>
+        </is>
+      </c>
+      <c r="H17" s="36" t="inlineStr">
+        <is>
+          <t>Il faudrait un suivi après ses formations par exemple qui a créé un agent IA depuis la formation dans son cadre mission ?
+Proposer de bloquer un créneau de 30 min avec Antho ou Matt et repartir avec un agent IA adapté au besoin d’un consultant en mission?</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="32">
-      <c r="C18" s="62" t="n"/>
-      <c r="F18" s="36" t="n"/>
-      <c r="G18" s="36" t="n"/>
-      <c r="H18" s="36" t="n"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>r-015</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>F-2026-004</t>
+        </is>
+      </c>
+      <c r="C18" s="63" t="n">
+        <v>46078.48716435185</v>
+      </c>
+      <c r="D18" t="n">
+        <v>5</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F18" s="36" t="inlineStr">
+        <is>
+          <t>Récupérer un assistant de prompt clé en main et pouvoir l'utiliser le jour-même.</t>
+        </is>
+      </c>
+      <c r="G18" s="36" t="inlineStr">
+        <is>
+          <t>Comme il s'agit d'un atelier très concret et actionnable : il serait pertinent de poursuivre l'exercice avec les formateurs, de façon plus personnalisée selon les besoins spécifiques des consultants.</t>
+        </is>
+      </c>
+      <c r="H18" s="36" t="inlineStr">
+        <is>
+          <t>Merci pour l'organisation de l'atelier :)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="32">
-      <c r="C19" s="62" t="n"/>
-      <c r="F19" s="36" t="n"/>
-      <c r="G19" s="36" t="n"/>
-      <c r="H19" s="36" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>r-016</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>F-2026-004</t>
+        </is>
+      </c>
+      <c r="C19" s="63" t="n">
+        <v>46078.4953587963</v>
+      </c>
+      <c r="D19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F19" s="36" t="inlineStr">
+        <is>
+          <t>rappel des différences entre assistant agent et agent agentique / recadrage sur les bonnes pratiques de prompt</t>
+        </is>
+      </c>
+      <c r="G19" s="36" t="inlineStr">
+        <is>
+          <t>sur l'exemple agent agentique vraiment insister sur le moment où le système est autonome. De manière très pratique à quelle moment le système fait des choses sans que j'ai besoin de le lancer pour qu'il les fasse</t>
+        </is>
+      </c>
+      <c r="H19" s="36" t="inlineStr">
+        <is>
+          <t>coeur sur vous</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="32">
-      <c r="C20" s="62" t="n"/>
-      <c r="F20" s="36" t="n"/>
-      <c r="G20" s="36" t="n"/>
-      <c r="H20" s="36" t="n"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>r-017</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>F-2026-004</t>
+        </is>
+      </c>
+      <c r="C20" s="63" t="n">
+        <v>46078.50295138889</v>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F20" s="36" t="inlineStr">
+        <is>
+          <t>La partie plus théorique, ça m'a permis de remettre les idées en place sur les RAG, assistants et agents</t>
+        </is>
+      </c>
+      <c r="G20" s="36" t="inlineStr">
+        <is>
+          <t>Je pense qu'il faudrait des sessions plus longues mais pas facile le soir</t>
+        </is>
+      </c>
+      <c r="H20" s="36" t="inlineStr">
+        <is>
+          <t>IXKO &lt;3</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="32">
-      <c r="C21" s="62" t="n"/>
-      <c r="F21" s="36" t="n"/>
-      <c r="G21" s="36" t="n"/>
-      <c r="H21" s="36" t="n"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>r-018</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>F-2026-004</t>
+        </is>
+      </c>
+      <c r="C21" s="63" t="n">
+        <v>46078.52372685185</v>
+      </c>
+      <c r="D21" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Oui mais j'ai besoin de plus de pratique</t>
+        </is>
+      </c>
+      <c r="F21" s="36" t="inlineStr">
+        <is>
+          <t>La partie pratique. Pouvoir manipuler les outils directement, ca permet de mieux se projeter dans l'utilisation quotidienne :)
+Découvrir les différences entre assistant, agent, ia agentique</t>
+        </is>
+      </c>
+      <c r="G21" s="36" t="inlineStr">
+        <is>
+          <t>Le passage sur le fonctionnement des systèmes de vecteurs mériterait d'être plus pédagogique ou illustré car c'est un concept clé qui est resté un peu flou
+Bien que la création d'un assistant ait été enrichissante, j'aurais aimé pousser la pratique jusqu'à la mise en place concrète d'un agent IA. Ca pourrait etre sympas de voir comment on passe d'un simple assistant conversationnel à un agent capable de planifier et d'exécuter des actions autonomes
+Pour fluidifier la partie pratique il serait préférable d'imposer un outil commun à tous les participants</t>
+        </is>
+      </c>
+      <c r="H21" s="36" t="inlineStr">
+        <is>
+          <t>bravo pour cette formation ! C'est une formation qui donne envie de creuser le sujet et d'expérimenter davantage</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="32">
-      <c r="C22" s="62" t="n"/>
-      <c r="F22" s="36" t="n"/>
-      <c r="G22" s="36" t="n"/>
-      <c r="H22" s="36" t="n"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>r-019</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>F-2026-004</t>
+        </is>
+      </c>
+      <c r="C22" s="63" t="n">
+        <v>46078.63008101852</v>
+      </c>
+      <c r="D22" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F22" s="36" t="inlineStr">
+        <is>
+          <t>Pas trop de théorie, de la place pour la pratique &amp; les échanges</t>
+        </is>
+      </c>
+      <c r="G22" s="36" t="inlineStr">
+        <is>
+          <t>Sur le fond et la forme pas de soucis
+L'horaire de la formation peut etre à discuter car en fin de journée on est un peu crevés
+On pourrait envisager un 13h/14h parfois ?</t>
+        </is>
+      </c>
+      <c r="H22" s="36" t="inlineStr">
+        <is>
+          <t>merci pour l'orga !</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="32">
-      <c r="C23" s="62" t="n"/>
-      <c r="F23" s="36" t="n"/>
-      <c r="G23" s="36" t="n"/>
-      <c r="H23" s="36" t="n"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>r-020</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>F-2026-004</t>
+        </is>
+      </c>
+      <c r="C23" s="63" t="n">
+        <v>46079.64048611111</v>
+      </c>
+      <c r="D23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F23" s="36" t="inlineStr">
+        <is>
+          <t>j'ai aimé le retour d'expérience sur le cas concret de l'agent pour la discovery</t>
+        </is>
+      </c>
+      <c r="G23" s="36" t="inlineStr">
+        <is>
+          <t>on aurait peut être pu faire un brainstorming pour des idées d'agents à créer, agents qui peuvent servir dans la vie quotidienne d'un PM =&gt; je trouve que ça peut nous donner des idées pour des futurs agents à créer</t>
+        </is>
+      </c>
+      <c r="H23" s="36" t="inlineStr">
+        <is>
+          <t>Je me demande si on ne pourrait pas se faire une bibliothèque partagée avec des prompts pour des agents qui nous servent au quotidien ? Merci pour la session en tous les cas !</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="32">
-      <c r="C24" s="62" t="n"/>
-      <c r="F24" s="36" t="n"/>
-      <c r="G24" s="36" t="n"/>
-      <c r="H24" s="36" t="n"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>r-021</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>F-2026-005</t>
+        </is>
+      </c>
+      <c r="C24" s="63" t="n">
+        <v>46099.42725694444</v>
+      </c>
+      <c r="D24" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Oui mais j'ai besoin de plus de pratique</t>
+        </is>
+      </c>
+      <c r="F24" s="36" t="inlineStr">
+        <is>
+          <t>Les explications claires, l'accompagnement et l'enchainement des étapes présentées par Théo + la pratique bien évidemment.</t>
+        </is>
+      </c>
+      <c r="G24" s="36" t="inlineStr">
+        <is>
+          <t>Attention au rythme, tout le monde ne va pas forcément à la même vitesse, ce qui ne facilite pas forcément la compréhension par moment.</t>
+        </is>
+      </c>
+      <c r="H24" s="36" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="32">
-      <c r="C25" s="62" t="n"/>
-      <c r="F25" s="36" t="n"/>
-      <c r="G25" s="36" t="n"/>
-      <c r="H25" s="36" t="n"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>r-022</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>F-2026-005</t>
+        </is>
+      </c>
+      <c r="C25" s="63" t="n">
+        <v>46099.43018518519</v>
+      </c>
+      <c r="D25" t="n">
+        <v>5</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Oui mais j'ai besoin de plus de pratique</t>
+        </is>
+      </c>
+      <c r="F25" s="36" t="inlineStr">
+        <is>
+          <t>La préparation et le cas pratique. Il y avait beaucoup de flexibilité pour répondre à un objectif simple. On avoisine quotidiennement ces notions et c'est bien d'enfin mettre le nez dedans</t>
+        </is>
+      </c>
+      <c r="G25" s="36" t="inlineStr">
+        <is>
+          <t>Sensibiliser par rapport à l'usage de l'IA et ses limites. Clairement j'en ai abusé pour customiser mon front et quand il s'agissait d'aller voir dans le code, très difficile. Peut-être ajouter des petites bonnes pratiques de vibe coding pour appliquer dans notre quotidien de PM (ce n'était pas le but de la formation)</t>
+        </is>
+      </c>
+      <c r="H25" s="36" t="inlineStr">
+        <is>
+          <t>Très hâte de la suite de ce parcours TechforPM</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="32">
-      <c r="C26" s="62" t="n"/>
-      <c r="F26" s="36" t="n"/>
-      <c r="G26" s="36" t="n"/>
-      <c r="H26" s="36" t="n"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>r-023</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>F-2026-005</t>
+        </is>
+      </c>
+      <c r="C26" s="63" t="n">
+        <v>46099.44282407407</v>
+      </c>
+      <c r="D26" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Oui mais j'ai besoin de plus de pratique</t>
+        </is>
+      </c>
+      <c r="F26" s="36" t="inlineStr">
+        <is>
+          <t>la mise en pratique = le fait de voir concrètement à quoi sert ce que nous manipulons</t>
+        </is>
+      </c>
+      <c r="G26" s="36" t="inlineStr">
+        <is>
+          <t>plus de contexte sur les commandes à faire dans le terminal = à quoi correspond cd, nps ..., plus de détails sur l'arborescence du front que nous créons pour bien comprendre pour quoi on créé tel variable à tel endroit</t>
+        </is>
+      </c>
+      <c r="H26" s="36" t="inlineStr">
+        <is>
+          <t>Merciiii</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="32">
-      <c r="C27" s="62" t="n"/>
-      <c r="F27" s="36" t="n"/>
-      <c r="G27" s="36" t="n"/>
-      <c r="H27" s="36" t="n"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>r-024</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>F-2026-005</t>
+        </is>
+      </c>
+      <c r="C27" s="63" t="n">
+        <v>46099.4693287037</v>
+      </c>
+      <c r="D27" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F27" s="36" t="inlineStr">
+        <is>
+          <t>Le projet d'acculturation technique mise en place par IKXO.</t>
+        </is>
+      </c>
+      <c r="G27" s="36" t="inlineStr">
+        <is>
+          <t>J'ai trouvé la marche bien trop haute pour une initiation. Le format "hands-on" immédiat sur trois outils complexes nécessite des bases que je n'avais pas, et m'a semblé plus adapté à des profils ayant déjà une sensibilité technique ou une formation d'ingénieur. J'ai rapidement décroché face à la complexité des instructions, ce qui a limité l'apport de la formation pour mon quotidien de PM. Il serait peut-être pertinent de segmenter les groupes par niveau ou de proposer une version plus 'théorique' pour comprendre les flux sans forcément manipuler le code.</t>
+        </is>
+      </c>
+      <c r="H27" s="36" t="inlineStr">
+        <is>
+          <t>Merci quand même à Théo et Jérém pour l"organisation</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="32">
-      <c r="C28" s="62" t="n"/>
-      <c r="F28" s="36" t="n"/>
-      <c r="G28" s="36" t="n"/>
-      <c r="H28" s="36" t="n"/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>r-025</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>F-2026-005</t>
+        </is>
+      </c>
+      <c r="C28" s="63" t="n">
+        <v>46099.51030092593</v>
+      </c>
+      <c r="D28" t="n">
+        <v>4</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Pas sûr</t>
+        </is>
+      </c>
+      <c r="F28" s="36" t="inlineStr">
+        <is>
+          <t>le côté travaux pratique avec Théo qui était très disponible pour chaque personne et chaque problématique (et j'ai bien galéré haha) sa maitrise du sujet qui donne vraiment envie de s'y intéresser et les parallèles fait avec les mots clés qu'on entend souvent d'un tech lead "merge request" "code review" "je vais merger ma branche" "rebase une branche" et où on sait pas exactement ce qu'il se passe derrière :)</t>
+        </is>
+      </c>
+      <c r="G28" s="36" t="inlineStr">
+        <is>
+          <t>Peut être une introduction plus générale et accessible pour réexpliquer les principes clés, la partie pratique est un point fort mais j'étais un peu perdue dans le déroulé des actions -&gt; peut être mettre sur les slides un avancement "étape 1 : blabla" un emoji "done" étape 2 : blabla" c'est là ou on en est et les étapes suivantes en grisées -&gt; cette frise nous suit sur tout l'avancement des étapes en haut des slides comme un résumé de ce qu'on a déjà fait et ce qu'il reste à faire
+Juste pour garder le recul sur ce qu'on est entrain de faire et où on en est car j'avais peu de maitrise sur les outils et les commandes donc même si Théo donnait du contexte à l'oral et des explications j'avais du mal à écouter et faire en même temps ce qui crée des décalages d'avancement chez les gens</t>
+        </is>
+      </c>
+      <c r="H28" s="36" t="inlineStr">
+        <is>
+          <t>Je trouve la formation super intéressante surtout grâce à la passion de Théo qui nous a partagé son projet perso aussi donc c'est très motivant et inspirant en revanche en tant que PM je ne sais pas trop si je peux appliquer ça directement dans mon travail de manière aussi opérationnelle mais par contre ça me donne une bonne vision de ce que y'a sous le capot de la machine et me donne du vocabulaire et de la compréhension poussée sur ce que font les développeurs :)</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="32">
-      <c r="C29" s="62" t="n"/>
-      <c r="F29" s="36" t="n"/>
-      <c r="G29" s="36" t="n"/>
-      <c r="H29" s="36" t="n"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>r-026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>F-2026-005</t>
+        </is>
+      </c>
+      <c r="C29" s="63" t="n">
+        <v>46099.75737268518</v>
+      </c>
+      <c r="D29" t="n">
+        <v>5</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Oui mais j'ai besoin de plus de pratique</t>
+        </is>
+      </c>
+      <c r="F29" s="36" t="inlineStr">
+        <is>
+          <t>Qu’on puisse très rapidement, mettre en pratique et voir les résultats !</t>
+        </is>
+      </c>
+      <c r="G29" s="36" t="inlineStr">
+        <is>
+          <t>La durée, 2h c’est assez court finalement pour se genre de travaux pratiques.
+Mais le soir je me doutes bien que c’est pas facile</t>
+        </is>
+      </c>
+      <c r="H29" s="36" t="inlineStr">
+        <is>
+          <t>Théo boss formateur ❤️🫰</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="32">
-      <c r="C30" s="62" t="n"/>
-      <c r="F30" s="36" t="n"/>
-      <c r="G30" s="36" t="n"/>
-      <c r="H30" s="36" t="n"/>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>r-027</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>F-2026-005</t>
+        </is>
+      </c>
+      <c r="C30" s="63" t="n">
+        <v>46099.81461805556</v>
+      </c>
+      <c r="D30" t="n">
+        <v>5</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Oui mais j'ai besoin de plus de pratique</t>
+        </is>
+      </c>
+      <c r="F30" s="36" t="inlineStr">
+        <is>
+          <t>J’ai bcp aimé le côté très pratique de la formation. On ne reste pas juste dans la théorie, on manipule directement les outils (VS Code, Git, GitHub, les branches, les merge, les PR…), ce qui aide vraiment à bien comprendre.
+Et franchement, c’est super intéressant d’apprendre des choses qui ne sont pas toujours faciles à trouver en ligne, même avec des formations payantes. Le fait de le voir à travers un cas simple et concret, ça rend tout beaucoup plus clair et utile pour notre métier.</t>
+        </is>
+      </c>
+      <c r="G30" s="36" t="inlineStr">
+        <is>
+          <t>Je pense qu’il faudrait un peu plus de temps entre les étapes. Par moments, le rythme est assez soutenu, et si on bloque au début, on peut vite perdre le fil et avoir du mal à suivre la suite. Un petit temps pour poser des questions ou vérifier que tout le monde a bien compris aiderait à ne pas décrocher.
+Aussi, parfois on doit recopier des informations affichées sur la presentation, si on a du retard, on peu rater ces éléments et vite etre dépassé sans moyen de reprendre le fil. On doit déranger Théo lors de sa pres ou déranger les autres pour rattraper. Ce serait plus pratique de recevoir les éléments directement (par exemple en amont ou via le canal formation) afin de pouvoir rattraper meme en solo</t>
+        </is>
+      </c>
+      <c r="H30" s="36" t="inlineStr">
+        <is>
+          <t>Un grand merci à Théo pour cette formation, elle était vraiment top et super intéressante. Franchement, ça va beaucoup m’aider dans la compréhension des outils et dans mon quotidien. C’est hyper appréciable d’avoir ce type de session en interne.
+J'ai hâte de voir la suite. C’est une super initiative et ça donne envie de progresser encore plus !
+Et si possible, ce serait top d’avoir un enregistrement ou un support pour pouvoir refaire les exercices ou rattraper une session en cas d’absence. Ça permettrait de ne rien perdre et de pouvoir revoir tranquillement les points abordés
+Julien</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="32">
-      <c r="C31" s="62" t="n"/>
-      <c r="F31" s="36" t="n"/>
-      <c r="G31" s="36" t="n"/>
-      <c r="H31" s="36" t="n"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>r-028</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>F-2026-005</t>
+        </is>
+      </c>
+      <c r="C31" s="63" t="n">
+        <v>46100.41905092593</v>
+      </c>
+      <c r="D31" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Pas sûr</t>
+        </is>
+      </c>
+      <c r="F31" s="36" t="inlineStr">
+        <is>
+          <t>La pratique</t>
+        </is>
+      </c>
+      <c r="G31" s="36" t="inlineStr">
+        <is>
+          <t>Pour ceux ayant des contraintes de PC dû au client cela n’a pas été optimal</t>
+        </is>
+      </c>
+      <c r="H31" s="36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="32">
-      <c r="C32" s="62" t="n"/>
-      <c r="F32" s="36" t="n"/>
-      <c r="G32" s="36" t="n"/>
-      <c r="H32" s="36" t="n"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>r-029</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>F-2026-005</t>
+        </is>
+      </c>
+      <c r="C32" s="63" t="n">
+        <v>46100.50283564815</v>
+      </c>
+      <c r="D32" t="n">
+        <v>5</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Oui mais j'ai besoin de plus de pratique</t>
+        </is>
+      </c>
+      <c r="F32" s="36" t="inlineStr">
+        <is>
+          <t>Tout, de la théorie à la pratique, c'était nickel</t>
+        </is>
+      </c>
+      <c r="G32" s="36" t="inlineStr">
+        <is>
+          <t>Déjà envoyé en MP à l'intéressé ;)</t>
+        </is>
+      </c>
+      <c r="H32" s="36" t="inlineStr">
+        <is>
+          <t>Vivement la prochaine</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="32">
-      <c r="C33" s="62" t="n"/>
-      <c r="F33" s="36" t="n"/>
-      <c r="G33" s="36" t="n"/>
-      <c r="H33" s="36" t="n"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>r-030</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>F-2026-006</t>
+        </is>
+      </c>
+      <c r="C33" s="63" t="n">
+        <v>46149.48512731482</v>
+      </c>
+      <c r="D33" t="n">
+        <v>4</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F33" s="36" t="inlineStr">
+        <is>
+          <t>J’ai bien aimé le rappel des points importants d’une roadmap et la présentation des différents formats. Ça permet de voir qu’en fonction de l’audience certains formats sont plus adaptés que d’autres.
+Le cas pratique à la fin était aussi super utile pour mieux retenir les choses et voir les points qu’on n’avait pas forcément bien compris.
+Les slides sont top :)</t>
+        </is>
+      </c>
+      <c r="G33" s="36" t="inlineStr">
+        <is>
+          <t>Peut-être qu’on pourrait aussi aborder la notion de priorisation, qui va vraiment de pair avec la roadmap. Je ne sais pas si c’est prévu dans une autre session de formation, mais ça serait intéressant de creuser ce sujet en complément.
+On n’a pas trop abordé la question des horizons de roadmap (3 mois, 6 mois, 1 an...), ca pourrait être intéressant d’avoir un peu plus de repères là-dessus.</t>
+        </is>
+      </c>
+      <c r="H33" s="36" t="inlineStr">
+        <is>
+          <t>Bravo et merci pour la formation ! c’était clair et utile. C’est toujours un plaisir d’y participer, on ressort avec des choses concrètes et directement réutilisables en mission.
+Julien</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="32">
-      <c r="C34" s="62" t="n"/>
-      <c r="F34" s="36" t="n"/>
-      <c r="G34" s="36" t="n"/>
-      <c r="H34" s="36" t="n"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>r-031</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>F-2026-006</t>
+        </is>
+      </c>
+      <c r="C34" s="63" t="n">
+        <v>46149.73609953704</v>
+      </c>
+      <c r="D34" t="n">
+        <v>5</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F34" s="36" t="inlineStr">
+        <is>
+          <t>Le cas pratique !!</t>
+        </is>
+      </c>
+      <c r="G34" s="36" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="H34" s="36" t="inlineStr">
+        <is>
+          <t>Au top :)</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="32">
-      <c r="C35" s="62" t="n"/>
-      <c r="F35" s="36" t="n"/>
-      <c r="G35" s="36" t="n"/>
-      <c r="H35" s="36" t="n"/>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>r-032</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>F-2026-006</t>
+        </is>
+      </c>
+      <c r="C35" s="63" t="n">
+        <v>46149.77533564815</v>
+      </c>
+      <c r="D35" t="n">
+        <v>5</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F35" s="36" t="inlineStr">
+        <is>
+          <t>Mise en pratique</t>
+        </is>
+      </c>
+      <c r="G35" s="36" t="inlineStr">
+        <is>
+          <t>Time management</t>
+        </is>
+      </c>
+      <c r="H35" s="36" t="inlineStr">
+        <is>
+          <t>merci beaucoup !</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="32">
-      <c r="C36" s="62" t="n"/>
-      <c r="F36" s="36" t="n"/>
-      <c r="G36" s="36" t="n"/>
-      <c r="H36" s="36" t="n"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>r-033</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>F-2026-006</t>
+        </is>
+      </c>
+      <c r="C36" s="63" t="n">
+        <v>46149.85436342593</v>
+      </c>
+      <c r="D36" t="n">
+        <v>5</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F36" s="36" t="inlineStr">
+        <is>
+          <t>Le cas d'usage</t>
+        </is>
+      </c>
+      <c r="G36" s="36" t="inlineStr">
+        <is>
+          <t>Expliciter les éléments à prendre en compte pour la construction de la roadmap ( pourcentage d'innovation etc) , dire en fonction de l'Organisation si telle ou telle roadmap est plus adaptée, donner des REX de consultants en mission</t>
+        </is>
+      </c>
+      <c r="H36" s="36" t="inlineStr">
+        <is>
+          <t>Mercii</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="32">
-      <c r="C37" s="62" t="n"/>
-      <c r="F37" s="36" t="n"/>
-      <c r="G37" s="36" t="n"/>
-      <c r="H37" s="36" t="n"/>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>r-034</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>F-2026-006</t>
+        </is>
+      </c>
+      <c r="C37" s="63" t="n">
+        <v>46153.43859953704</v>
+      </c>
+      <c r="D37" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F37" s="36" t="inlineStr">
+        <is>
+          <t>Le mix connaissance/application, ainsi que la qualité des informations données</t>
+        </is>
+      </c>
+      <c r="G37" s="36" t="inlineStr">
+        <is>
+          <t>un peu plus d'exemples concrets même s'il y en avait déjà</t>
+        </is>
+      </c>
+      <c r="H37" s="36" t="inlineStr">
+        <is>
+          <t>J'ai beaucoup apprécié la session ! Merci encore</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="32">
-      <c r="C38" s="62" t="n"/>
-      <c r="F38" s="36" t="n"/>
-      <c r="G38" s="36" t="n"/>
-      <c r="H38" s="36" t="n"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>r-035</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>F-2026-006</t>
+        </is>
+      </c>
+      <c r="C38" s="63" t="n">
+        <v>46153.44553240741</v>
+      </c>
+      <c r="D38" t="n">
+        <v>5</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F38" s="36" t="inlineStr">
+        <is>
+          <t>Les exemples concrets</t>
+        </is>
+      </c>
+      <c r="G38" s="36" t="inlineStr">
+        <is>
+          <t>Avoir plus de temps pour la pratique</t>
+        </is>
+      </c>
+      <c r="H38" s="36" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="32">
-      <c r="C39" s="62" t="n"/>
-      <c r="F39" s="36" t="n"/>
-      <c r="G39" s="36" t="n"/>
-      <c r="H39" s="36" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>r-036</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>F-2026-006</t>
+        </is>
+      </c>
+      <c r="C39" s="63" t="n">
+        <v>46155.67434027778</v>
+      </c>
+      <c r="D39" t="n">
+        <v>5</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F39" s="36" t="inlineStr">
+        <is>
+          <t>La reprise des bases mais surtout que ce soit applicable/transférable à la mission</t>
+        </is>
+      </c>
+      <c r="G39" s="36" t="inlineStr">
+        <is>
+          <t>une assiette de cookies tout chaud ce serait du luxe mais sinon j'ai trouvé ça top !</t>
+        </is>
+      </c>
+      <c r="H39" s="36" t="inlineStr">
+        <is>
+          <t>c'était ni trop léger, ni trop chargé. Au top pour tout assimiler. Je pense que tu as surestimé le temps pour l'exercice, les points qu'on a fait étaient suffisants pour bien maitriser la notion</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="32">
-      <c r="C40" s="62" t="n"/>
-      <c r="F40" s="36" t="n"/>
-      <c r="G40" s="36" t="n"/>
-      <c r="H40" s="36" t="n"/>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>r-037</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>F-2026-007</t>
+        </is>
+      </c>
+      <c r="C40" s="63" t="n">
+        <v>46120.41951388889</v>
+      </c>
+      <c r="D40" t="n">
+        <v>5</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F40" s="36" t="inlineStr">
+        <is>
+          <t>Anthony est bon pour garder notre attention je trouve :)</t>
+        </is>
+      </c>
+      <c r="G40" s="36" t="inlineStr">
+        <is>
+          <t>Plus de pratique (mais en même temps on voulais tous terminer à 19h donc compliqué … à la limite commencer un peu plus tôt)</t>
+        </is>
+      </c>
+      <c r="H40" s="36" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="32">
-      <c r="C41" s="62" t="n"/>
-      <c r="F41" s="36" t="n"/>
-      <c r="G41" s="36" t="n"/>
-      <c r="H41" s="36" t="n"/>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>r-038</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>F-2026-007</t>
+        </is>
+      </c>
+      <c r="C41" s="63" t="n">
+        <v>46120.4254050926</v>
+      </c>
+      <c r="D41" t="n">
+        <v>4</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F41" s="36" t="inlineStr">
+        <is>
+          <t>Bonne animation d'Antho, un mix formation et discussion informelle appuyée par des exemples concrets en mission</t>
+        </is>
+      </c>
+      <c r="G41" s="36" t="inlineStr">
+        <is>
+          <t>Si je veux vraiment être tatillon, avoir un jeu de données prêt à l'emploi (et peut être dire concrètement lequel utilise et comment l'utiliser)</t>
+        </is>
+      </c>
+      <c r="H41" s="36" t="inlineStr">
+        <is>
+          <t>Super formation, 1H sharp, pas trop lourd et pas inutile. Merci à Antho ! (et Matt même si il est en trian de chasser les fantômes en Ecosse)</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="32">
-      <c r="C42" s="62" t="n"/>
-      <c r="F42" s="36" t="n"/>
-      <c r="G42" s="36" t="n"/>
-      <c r="H42" s="36" t="n"/>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>r-039</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>F-2026-007</t>
+        </is>
+      </c>
+      <c r="C42" s="63" t="n">
+        <v>46120.4412962963</v>
+      </c>
+      <c r="D42" t="n">
+        <v>5</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F42" s="36" t="inlineStr">
+        <is>
+          <t>Partie pratique</t>
+        </is>
+      </c>
+      <c r="G42" s="36" t="inlineStr">
+        <is>
+          <t>Aucun, c'était synthétique &amp; efficace</t>
+        </is>
+      </c>
+      <c r="H42" s="36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="32">
-      <c r="C43" s="62" t="n"/>
-      <c r="F43" s="36" t="n"/>
-      <c r="G43" s="36" t="n"/>
-      <c r="H43" s="36" t="n"/>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>r-040</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>F-2026-007</t>
+        </is>
+      </c>
+      <c r="C43" s="63" t="n">
+        <v>46120.4891087963</v>
+      </c>
+      <c r="D43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F43" s="36" t="inlineStr">
+        <is>
+          <t>Mise en pratique</t>
+        </is>
+      </c>
+      <c r="G43" s="36" t="inlineStr">
+        <is>
+          <t>Faire sur le midi plutôt que le soir, car on s’entait que tout le monde avait envie de rentrer chez soi.</t>
+        </is>
+      </c>
+      <c r="H43" s="36" t="inlineStr">
+        <is>
+          <t>Merci 🙏</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="32">
-      <c r="C44" s="62" t="n"/>
-      <c r="F44" s="36" t="n"/>
-      <c r="G44" s="36" t="n"/>
-      <c r="H44" s="36" t="n"/>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>r-041</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>F-2026-007</t>
+        </is>
+      </c>
+      <c r="C44" s="63" t="n">
+        <v>46120.52988425926</v>
+      </c>
+      <c r="D44" t="n">
+        <v>5</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F44" s="36" t="inlineStr">
+        <is>
+          <t>La mise en pratique immédiate</t>
+        </is>
+      </c>
+      <c r="G44" s="36" t="inlineStr">
+        <is>
+          <t>La présentation des slides était un peu brouillon. Certaines slides répétaient la précédente. Ca ne m’a pas dérangé car nous sommes entre nous mais il faut bien trouver un axe.</t>
+        </is>
+      </c>
+      <c r="H44" s="36" t="inlineStr">
+        <is>
+          <t>Très content de cette première formation chez XO. J’ai eu l’impression que ça a duré 5 minutes.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="32">
-      <c r="C45" s="62" t="n"/>
-      <c r="F45" s="36" t="n"/>
-      <c r="G45" s="36" t="n"/>
-      <c r="H45" s="36" t="n"/>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>r-042</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>F-2026-007</t>
+        </is>
+      </c>
+      <c r="C45" s="63" t="n">
+        <v>46120.57973379629</v>
+      </c>
+      <c r="D45" t="n">
+        <v>5</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F45" s="36" t="inlineStr">
+        <is>
+          <t>Le cas pratique</t>
+        </is>
+      </c>
+      <c r="G45" s="36" t="inlineStr">
+        <is>
+          <t>Cas pratique plus poussé avec un cas mission</t>
+        </is>
+      </c>
+      <c r="H45" s="36" t="inlineStr">
+        <is>
+          <t>All good !</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="32">
-      <c r="C46" s="62" t="n"/>
-      <c r="F46" s="36" t="n"/>
-      <c r="G46" s="36" t="n"/>
-      <c r="H46" s="36" t="n"/>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>r-043</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>F-2026-008</t>
+        </is>
+      </c>
+      <c r="C46" s="63" t="n">
+        <v>46141.47037037037</v>
+      </c>
+      <c r="D46" t="n">
+        <v>5</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Pas sûr</t>
+        </is>
+      </c>
+      <c r="F46" s="36" t="inlineStr">
+        <is>
+          <t>ça nous permet d'appréhender la manière dont travaillent les techs + les complexités associées</t>
+        </is>
+      </c>
+      <c r="G46" s="36" t="inlineStr">
+        <is>
+          <t>Il faut peut etre envisager de faire des groupes de niveaux et adapter le scope en fonction
+Certaines personnes déjà à l'aise avec ces outils avaient largement fini et d'autres comme moi on mis au moins 2H/2H15</t>
+        </is>
+      </c>
+      <c r="H46" s="36" t="inlineStr">
+        <is>
+          <t>sujet super intéréssant</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="32">
-      <c r="C47" s="62" t="n"/>
-      <c r="F47" s="36" t="n"/>
-      <c r="G47" s="36" t="n"/>
-      <c r="H47" s="36" t="n"/>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>r-044</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>F-2026-008</t>
+        </is>
+      </c>
+      <c r="C47" s="63" t="n">
+        <v>46141.47042824074</v>
+      </c>
+      <c r="D47" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Oui immédiatement</t>
+        </is>
+      </c>
+      <c r="F47" s="36" t="inlineStr">
+        <is>
+          <t>La pratique 💜</t>
+        </is>
+      </c>
+      <c r="G47" s="36" t="inlineStr">
+        <is>
+          <t>Bah les formations techniques demandent plus de temps donc dans l’idéal on aurait du commencer à 17h pour bien avoir le temps de tout faire</t>
+        </is>
+      </c>
+      <c r="H47" s="36" t="inlineStr">
+        <is>
+          <t>Commencer les formation lus tôt 17h 😆</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="32">
-      <c r="C48" s="62" t="n"/>
-      <c r="F48" s="36" t="n"/>
-      <c r="G48" s="36" t="n"/>
-      <c r="H48" s="36" t="n"/>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>r-045</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>F-2026-008</t>
+        </is>
+      </c>
+      <c r="C48" s="63" t="n">
+        <v>46141.47488425926</v>
+      </c>
+      <c r="D48" t="n">
+        <v>5</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Pas sûr</t>
+        </is>
+      </c>
+      <c r="F48" s="36" t="inlineStr">
+        <is>
+          <t>deep into tech. mieux comprendre le quotidien de mes devs</t>
+        </is>
+      </c>
+      <c r="G48" s="36" t="inlineStr">
+        <is>
+          <t>timing de la session. il faut plus de temps</t>
+        </is>
+      </c>
+      <c r="H48" s="36" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="32">
-      <c r="C49" s="62" t="n"/>
-      <c r="F49" s="36" t="n"/>
-      <c r="G49" s="36" t="n"/>
-      <c r="H49" s="36" t="n"/>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>r-046</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>F-2026-008</t>
+        </is>
+      </c>
+      <c r="C49" s="63" t="n">
+        <v>46142.54083333333</v>
+      </c>
+      <c r="D49" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Oui mais j'ai besoin de plus de pratique</t>
+        </is>
+      </c>
+      <c r="F49" s="36" t="inlineStr">
+        <is>
+          <t>La disponibilité des formateurs, l'ambiance de travail et la découverte du sujet</t>
+        </is>
+      </c>
+      <c r="G49" s="36" t="inlineStr">
+        <is>
+          <t>Tout dépend ce que l'on souhaite faire mais soit il faut rendre la session plus didactique (montrer ce qu'on doit faire pas à pas) ou alors pas d'amélioration et on garde cet esprit plus de découverte et d'exploration (ce qui peut amener à des erreurs. Ex : un dossier initial mal enregistré qui pose un pb dans la génération du code)
+Quelques cheat-sheets en 2-pager auraient été cool je pense.
+Autre aspect, je me suis demandé si Theo/Simon arrivaient réellement à savoir ou chaque personne étaient rendues. Je me suis dit qu'avoir un board de "check-in" pourrait être pratique pour le suivi.
+Avoir un temps de réalisation pour chaque tâche aussi (au travers de la cheat-sheet) et qui soit raisonnable pour des novices</t>
+        </is>
+      </c>
+      <c r="H49" s="36" t="inlineStr">
+        <is>
+          <t>Nous n'avons pas pu tout faire de ce qui était prévu, ça serait cool de le dire soit au début soit à la fin de comment ça se passe dans ce cas.
+Dernier point, la session prend 2h (estimé 1h30 je crois). Il faut peut-être partir dans l'idée que dès le départ, nous nous arrêterons à 20h, quoi qui se passe.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="32">
-      <c r="C50" s="62" t="n"/>
-      <c r="F50" s="36" t="n"/>
-      <c r="G50" s="36" t="n"/>
-      <c r="H50" s="36" t="n"/>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>r-047</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>F-2026-008</t>
+        </is>
+      </c>
+      <c r="C50" s="63" t="n">
+        <v>46146.54844907407</v>
+      </c>
+      <c r="D50" t="n">
+        <v>2</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F50" s="36" t="inlineStr">
+        <is>
+          <t>L’aide de Théo lors d’un blocage</t>
+        </is>
+      </c>
+      <c r="G50" s="36" t="inlineStr">
+        <is>
+          <t>Expliquer pourquoi on utilise cette commande. J’ai suivi le guide mais sans comprendre pourquoi il fallait faire les actions.</t>
+        </is>
+      </c>
+      <c r="H50" s="36" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="32">
       <c r="C51" s="62" t="n"/>

</xml_diff>

<commit_message>
Mise a jour presences <mois> 2026
</commit_message>
<xml_diff>
--- a/public/data/suivi_presence_consultants.xlsx
+++ b/public/data/suivi_presence_consultants.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeremiekieffer/Projets/ikxo-presence-dashboard/public/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6FC2E581-CAED-C941-AA9B-8713EA1472FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{857BF823-69D5-D340-86CF-76CAF867E7EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-51200" yWindow="-1880" windowWidth="51200" windowHeight="27260" tabRatio="500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1053" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1063" uniqueCount="392">
   <si>
     <t>Convention de saisie — Suivi de présence consultants</t>
   </si>
@@ -3397,19 +3397,19 @@
       </c>
       <c r="C10" s="2">
         <f>SUM('Saisie 2026-06'!X4:X30)</f>
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="D10" s="2">
         <f>IFERROR(COUNTIF('Saisie 2026-06'!Y4:Y30,"Atteint")/(COUNTIF('Saisie 2026-06'!Y4:Y30,"Atteint")+COUNTIF('Saisie 2026-06'!Y4:Y30,"Sous objectif")),0)</f>
-        <v>7.6923076923076927E-2</v>
+        <v>0.30769230769230771</v>
       </c>
       <c r="E10" s="2">
         <f>IFERROR(SUM('Saisie 2026-06'!X4:X30)/(COUNTIF('Saisie 2026-06'!Y4:Y30,"Atteint")+COUNTIF('Saisie 2026-06'!Y4:Y30,"Sous objectif")),0)</f>
-        <v>0.57692307692307687</v>
+        <v>1.3461538461538463</v>
       </c>
       <c r="F10" s="2">
         <f>COUNTIF('Saisie 2026-06'!X4:X30,"&gt;=1")</f>
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>186</v>
@@ -3425,19 +3425,19 @@
       </c>
       <c r="C11" s="2">
         <f>AVERAGE(C8:C10)</f>
-        <v>59.333333333333336</v>
+        <v>66</v>
       </c>
       <c r="D11" s="2">
         <f>AVERAGE(D8:D10)</f>
-        <v>0.48717948717948717</v>
+        <v>0.5641025641025641</v>
       </c>
       <c r="E11" s="2">
         <f>AVERAGE(E8:E10)</f>
-        <v>2.2820512820512819</v>
+        <v>2.5384615384615383</v>
       </c>
       <c r="F11" s="2">
         <f>AVERAGE(F8:F10)</f>
-        <v>20.666666666666668</v>
+        <v>22.333333333333332</v>
       </c>
     </row>
   </sheetData>
@@ -3509,7 +3509,7 @@
       </c>
       <c r="F6" s="2">
         <f>IF('Saisie 2026-06'!Y4="N/A absence longue","M",'Saisie 2026-06'!X4)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="2">
         <f t="shared" ref="G6:G31" si="0">COUNTIF(B6:F6,"&gt;=2")</f>
@@ -3542,7 +3542,7 @@
       </c>
       <c r="F7" s="2">
         <f>IF('Saisie 2026-06'!Y5="N/A absence longue","M",'Saisie 2026-06'!X5)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G7" s="2">
         <f t="shared" si="0"/>
@@ -3608,15 +3608,15 @@
       </c>
       <c r="F9" s="2">
         <f>IF('Saisie 2026-06'!Y7="N/A absence longue","M",'Saisie 2026-06'!X7)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G9" s="2">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H9" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>4/5</v>
+        <v>5/5 ✓</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
@@ -3707,15 +3707,15 @@
       </c>
       <c r="F12" s="2">
         <f>IF('Saisie 2026-06'!Y11="N/A absence longue","M",'Saisie 2026-06'!X11)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G12" s="2">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H12" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>4/5</v>
+        <v>5/5 ✓</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="F15" s="2">
         <f>IF('Saisie 2026-06'!Y14="N/A absence longue","M",'Saisie 2026-06'!X14)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" s="2">
         <f t="shared" si="0"/>
@@ -3839,15 +3839,15 @@
       </c>
       <c r="F16" s="2">
         <f>IF('Saisie 2026-06'!Y15="N/A absence longue","M",'Saisie 2026-06'!X15)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G16" s="2">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H16" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>3/5</v>
+        <v>4/5</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="15.75" customHeight="1">
@@ -3872,15 +3872,15 @@
       </c>
       <c r="F17" s="2">
         <f>IF('Saisie 2026-06'!Y16="N/A absence longue","M",'Saisie 2026-06'!X16)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G17" s="2">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H17" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>4/5</v>
+        <v>5/5 ✓</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="15.75" customHeight="1">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="F19" s="2">
         <f>IF('Saisie 2026-06'!Y18="N/A absence longue","M",'Saisie 2026-06'!X18)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G19" s="2">
         <f t="shared" si="0"/>
@@ -4037,15 +4037,15 @@
       </c>
       <c r="F22" s="2">
         <f>IF('Saisie 2026-06'!Y21="N/A absence longue","M",'Saisie 2026-06'!X21)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" s="2">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H22" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>3/5</v>
+        <v>4/5</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="15.75" customHeight="1">
@@ -4070,15 +4070,15 @@
       </c>
       <c r="F23" s="2">
         <f>IF('Saisie 2026-06'!Y22="N/A absence longue","M",'Saisie 2026-06'!X22)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G23" s="2">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H23" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>4/5</v>
+        <v>5/5 ✓</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="15.75" customHeight="1">
@@ -4268,7 +4268,7 @@
       </c>
       <c r="F29" s="2">
         <f>IF('Saisie 2026-06'!Y28="N/A absence longue","M",'Saisie 2026-06'!X28)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" s="2">
         <f t="shared" si="0"/>
@@ -4301,7 +4301,7 @@
       </c>
       <c r="F30" s="2">
         <f>IF('Saisie 2026-06'!Y29="N/A absence longue","M",'Saisie 2026-06'!X29)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" s="2">
         <f t="shared" si="0"/>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="F31" s="2">
         <f>IF('Saisie 2026-06'!Y30="N/A absence longue","M",'Saisie 2026-06'!X30)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G31" s="2">
         <f t="shared" si="0"/>
@@ -11431,6 +11431,9 @@
       <c r="A10" s="2" t="s">
         <v>84</v>
       </c>
+      <c r="C10" s="6">
+        <v>46178</v>
+      </c>
     </row>
     <row r="11" spans="1:4" ht="15.75" customHeight="1">
       <c r="A11" s="2" t="s">
@@ -16893,7 +16896,9 @@
       <c r="E4" s="15"/>
       <c r="F4" s="14"/>
       <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
+      <c r="H4" s="14">
+        <v>1</v>
+      </c>
       <c r="I4" s="14"/>
       <c r="J4" s="15"/>
       <c r="K4" s="14"/>
@@ -16911,7 +16916,7 @@
       <c r="W4" s="14"/>
       <c r="X4" s="17">
         <f>COUNTIF(B4:W4,1)+COUNTIF(B4:W4,"IC")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y4" s="14" t="str">
         <f>IF(COUNTIF(B4:W4,"M")&gt;0,"N/A absence longue",IF(X4&gt;=2,"Atteint","Sous objectif"))</f>
@@ -16933,10 +16938,16 @@
         <v>9</v>
       </c>
       <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
+      <c r="G5" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>9</v>
+      </c>
       <c r="I5" s="14"/>
-      <c r="J5" s="15"/>
+      <c r="J5" s="15" t="s">
+        <v>9</v>
+      </c>
       <c r="K5" s="14"/>
       <c r="L5" s="14"/>
       <c r="M5" s="14"/>
@@ -16952,7 +16963,7 @@
       <c r="W5" s="14"/>
       <c r="X5" s="17">
         <f>COUNTIF(B5:W5,1)+COUNTIF(B5:W5,"IC")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Y5" s="14" t="str">
         <f>IF(COUNTIF(B5:W5,"M")&gt;0,"N/A absence longue",IF(X5&gt;=2,"Atteint","Sous objectif"))</f>
@@ -17006,9 +17017,13 @@
       <c r="E7" s="15"/>
       <c r="F7" s="14"/>
       <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
+      <c r="H7" s="14">
+        <v>1</v>
+      </c>
       <c r="I7" s="14"/>
-      <c r="J7" s="15"/>
+      <c r="J7" s="15">
+        <v>1</v>
+      </c>
       <c r="K7" s="14"/>
       <c r="L7" s="14"/>
       <c r="M7" s="14"/>
@@ -17024,11 +17039,11 @@
       <c r="W7" s="14"/>
       <c r="X7" s="17">
         <f>COUNTIF(B7:W7,1)+COUNTIF(B7:W7,"IC")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Y7" s="14" t="str">
         <f>IF(COUNTIF(B7:W7,"M")&gt;0,"N/A absence longue",IF(X7&gt;=2,"Atteint","Sous objectif"))</f>
-        <v>Sous objectif</v>
+        <v>Atteint</v>
       </c>
     </row>
     <row r="8" spans="1:25" ht="18" customHeight="1">
@@ -17048,10 +17063,16 @@
         <v>9</v>
       </c>
       <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="G8" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>9</v>
+      </c>
       <c r="I8" s="14"/>
-      <c r="J8" s="15"/>
+      <c r="J8" s="15" t="s">
+        <v>9</v>
+      </c>
       <c r="K8" s="14"/>
       <c r="L8" s="14"/>
       <c r="M8" s="14"/>
@@ -17154,9 +17175,13 @@
       </c>
       <c r="F11" s="14"/>
       <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
+      <c r="H11" s="14">
+        <v>1</v>
+      </c>
       <c r="I11" s="14"/>
-      <c r="J11" s="15"/>
+      <c r="J11" s="15">
+        <v>1</v>
+      </c>
       <c r="K11" s="14"/>
       <c r="L11" s="14"/>
       <c r="M11" s="14"/>
@@ -17172,11 +17197,11 @@
       <c r="W11" s="14"/>
       <c r="X11" s="17">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Y11" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>Sous objectif</v>
+        <v>Atteint</v>
       </c>
     </row>
     <row r="12" spans="1:25" ht="18" customHeight="1">
@@ -17260,7 +17285,9 @@
       <c r="D14" s="14"/>
       <c r="E14" s="15"/>
       <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
+      <c r="G14" s="14">
+        <v>1</v>
+      </c>
       <c r="H14" s="14"/>
       <c r="I14" s="14"/>
       <c r="J14" s="15"/>
@@ -17279,7 +17306,7 @@
       <c r="W14" s="14"/>
       <c r="X14" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y14" s="14" t="str">
         <f t="shared" si="1"/>
@@ -17298,7 +17325,9 @@
       <c r="E15" s="15"/>
       <c r="F15" s="14"/>
       <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
+      <c r="H15" s="14">
+        <v>1</v>
+      </c>
       <c r="I15" s="14"/>
       <c r="J15" s="15"/>
       <c r="K15" s="14"/>
@@ -17316,11 +17345,11 @@
       <c r="W15" s="14"/>
       <c r="X15" s="17">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y15" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>Sous objectif</v>
+        <v>Atteint</v>
       </c>
     </row>
     <row r="16" spans="1:25" ht="18" customHeight="1">
@@ -17335,7 +17364,9 @@
       <c r="E16" s="15"/>
       <c r="F16" s="14"/>
       <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
+      <c r="H16" s="14">
+        <v>1</v>
+      </c>
       <c r="I16" s="14"/>
       <c r="J16" s="15"/>
       <c r="K16" s="14"/>
@@ -17353,11 +17384,11 @@
       <c r="W16" s="14"/>
       <c r="X16" s="17">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y16" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>Sous objectif</v>
+        <v>Atteint</v>
       </c>
     </row>
     <row r="17" spans="1:25" ht="18" customHeight="1">
@@ -17408,10 +17439,16 @@
         <v>9</v>
       </c>
       <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
+      <c r="G18" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>9</v>
+      </c>
       <c r="I18" s="14"/>
-      <c r="J18" s="15"/>
+      <c r="J18" s="15" t="s">
+        <v>9</v>
+      </c>
       <c r="K18" s="14"/>
       <c r="L18" s="14"/>
       <c r="M18" s="14"/>
@@ -17427,7 +17464,7 @@
       <c r="W18" s="14"/>
       <c r="X18" s="17">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Y18" s="14" t="str">
         <f t="shared" si="1"/>
@@ -17515,7 +17552,9 @@
       <c r="D21" s="14"/>
       <c r="E21" s="15"/>
       <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
+      <c r="G21" s="14">
+        <v>1</v>
+      </c>
       <c r="H21" s="14"/>
       <c r="I21" s="14"/>
       <c r="J21" s="15"/>
@@ -17534,11 +17573,11 @@
       <c r="W21" s="14"/>
       <c r="X21" s="17">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y21" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>Sous objectif</v>
+        <v>Atteint</v>
       </c>
     </row>
     <row r="22" spans="1:25" ht="18" customHeight="1">
@@ -17551,9 +17590,13 @@
       <c r="E22" s="15">
         <v>1</v>
       </c>
-      <c r="F22" s="14"/>
+      <c r="F22" s="14">
+        <v>1</v>
+      </c>
       <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
+      <c r="H22" s="14">
+        <v>1</v>
+      </c>
       <c r="I22" s="14"/>
       <c r="J22" s="15"/>
       <c r="K22" s="14"/>
@@ -17571,11 +17614,11 @@
       <c r="W22" s="14"/>
       <c r="X22" s="17">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Y22" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>Sous objectif</v>
+        <v>Atteint</v>
       </c>
     </row>
     <row r="23" spans="1:25" ht="18" customHeight="1">
@@ -17765,7 +17808,9 @@
       <c r="E28" s="15"/>
       <c r="F28" s="14"/>
       <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
+      <c r="H28" s="14">
+        <v>1</v>
+      </c>
       <c r="I28" s="14"/>
       <c r="J28" s="15"/>
       <c r="K28" s="14"/>
@@ -17783,7 +17828,7 @@
       <c r="W28" s="14"/>
       <c r="X28" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y28" s="14" t="str">
         <f t="shared" si="1"/>
@@ -17800,7 +17845,9 @@
       <c r="E29" s="15"/>
       <c r="F29" s="14"/>
       <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
+      <c r="H29" s="14">
+        <v>1</v>
+      </c>
       <c r="I29" s="14"/>
       <c r="J29" s="15"/>
       <c r="K29" s="14"/>
@@ -17818,7 +17865,7 @@
       <c r="W29" s="14"/>
       <c r="X29" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y29" s="14" t="str">
         <f t="shared" si="1"/>
@@ -17835,7 +17882,9 @@
       <c r="E30" s="15"/>
       <c r="F30" s="14"/>
       <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
+      <c r="H30" s="14">
+        <v>1</v>
+      </c>
       <c r="I30" s="14"/>
       <c r="J30" s="15"/>
       <c r="K30" s="14"/>
@@ -17853,7 +17902,7 @@
       <c r="W30" s="14"/>
       <c r="X30" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y30" s="14" t="str">
         <f t="shared" si="1"/>
@@ -17902,7 +17951,9 @@
       <c r="E34" s="15"/>
       <c r="F34" s="14"/>
       <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
+      <c r="H34" s="14" t="s">
+        <v>18</v>
+      </c>
       <c r="I34" s="14"/>
       <c r="J34" s="15"/>
       <c r="K34" s="14"/>

</xml_diff>

<commit_message>
Mise a jour formations <mois> 2026
</commit_message>
<xml_diff>
--- a/public/data/suivi_presence_consultants.xlsx
+++ b/public/data/suivi_presence_consultants.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeremiekieffer/Projets/ikxo-presence-dashboard/public/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD457149-F2A2-674E-A456-327096DDAF34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E89EBFD8-7396-4D4D-B94C-F02542D0E4C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17520" tabRatio="500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17520" tabRatio="500" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Convention" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="397">
   <si>
     <t>Convention de saisie — Suivi de présence consultants</t>
   </si>
@@ -1272,6 +1272,18 @@
   </si>
   <si>
     <t>mu</t>
+  </si>
+  <si>
+    <t>F-2026-010</t>
+  </si>
+  <si>
+    <t>06/30/2026</t>
+  </si>
+  <si>
+    <t>Tech For PM#3 - Data Model</t>
+  </si>
+  <si>
+    <t>Théo Esposito, Geoffroy Debellabre</t>
   </si>
 </sst>
 </file>
@@ -1283,7 +1295,7 @@
     <numFmt numFmtId="165" formatCode="[$-40C]ddd\ dd"/>
     <numFmt numFmtId="166" formatCode="m/d/yyyy\ h:mm"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1349,6 +1361,12 @@
       <color rgb="FF6E7480"/>
       <name val="Cambria"/>
       <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -1448,7 +1466,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1523,11 +1541,28 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="29">
+  <dxfs count="31">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD1FAE5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2421,6 +2456,9 @@
       <c r="T3" s="8" t="s">
         <v>166</v>
       </c>
+      <c r="U3" s="32" t="s">
+        <v>393</v>
+      </c>
     </row>
     <row r="4" spans="1:27" ht="15" customHeight="1">
       <c r="A4" s="13" t="s">
@@ -2479,7 +2517,7 @@
       </c>
       <c r="B7" s="17">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D7" t="s">
         <v>33</v>
@@ -2509,6 +2547,9 @@
         <v>33</v>
       </c>
       <c r="T7" t="s">
+        <v>33</v>
+      </c>
+      <c r="U7" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2572,7 +2613,7 @@
       </c>
       <c r="B10" s="17">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -2605,6 +2646,9 @@
         <v>33</v>
       </c>
       <c r="T10" t="s">
+        <v>33</v>
+      </c>
+      <c r="U10" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2614,7 +2658,10 @@
       </c>
       <c r="B11" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="U11" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:27" ht="15" customHeight="1">
@@ -2656,7 +2703,7 @@
       </c>
       <c r="B14" s="17">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K14" t="s">
         <v>33</v>
@@ -2665,6 +2712,9 @@
         <v>30</v>
       </c>
       <c r="S14" t="s">
+        <v>30</v>
+      </c>
+      <c r="U14" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2674,7 +2724,7 @@
       </c>
       <c r="B15" s="17">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C15" t="s">
         <v>33</v>
@@ -2692,6 +2742,9 @@
         <v>33</v>
       </c>
       <c r="S15" t="s">
+        <v>33</v>
+      </c>
+      <c r="U15" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2701,7 +2754,7 @@
       </c>
       <c r="B16" s="17">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K16" t="s">
         <v>33</v>
@@ -2721,14 +2774,17 @@
       <c r="T16" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="17" spans="1:20" ht="15" customHeight="1">
+      <c r="U16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" ht="15" customHeight="1">
       <c r="A17" s="13" t="s">
         <v>86</v>
       </c>
       <c r="B17" s="17">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E17" t="s">
         <v>33</v>
@@ -2742,14 +2798,17 @@
       <c r="R17" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="18" spans="1:20" ht="15" customHeight="1">
+      <c r="U17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" ht="15" customHeight="1">
       <c r="A18" s="13" t="s">
         <v>92</v>
       </c>
       <c r="B18" s="17">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J18" t="s">
         <v>33</v>
@@ -2763,8 +2822,11 @@
       <c r="R18" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="19" spans="1:20" ht="15" customHeight="1">
+      <c r="U18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" ht="15" customHeight="1">
       <c r="A19" s="13" t="s">
         <v>100</v>
       </c>
@@ -2800,7 +2862,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="15" customHeight="1">
+    <row r="20" spans="1:21" ht="15" customHeight="1">
       <c r="A20" s="13" t="s">
         <v>91</v>
       </c>
@@ -2824,7 +2886,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="15" customHeight="1">
+    <row r="21" spans="1:21" ht="15" customHeight="1">
       <c r="A21" s="13" t="s">
         <v>83</v>
       </c>
@@ -2845,7 +2907,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="15" customHeight="1">
+    <row r="22" spans="1:21" ht="15" customHeight="1">
       <c r="A22" s="13" t="s">
         <v>84</v>
       </c>
@@ -2869,7 +2931,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="15" customHeight="1">
+    <row r="23" spans="1:21" ht="15" customHeight="1">
       <c r="A23" s="13" t="s">
         <v>80</v>
       </c>
@@ -2893,19 +2955,22 @@
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:20" ht="15" customHeight="1">
+    <row r="24" spans="1:21" ht="15" customHeight="1">
       <c r="A24" s="13" t="s">
         <v>87</v>
       </c>
       <c r="B24" s="17">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q24" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="25" spans="1:20" ht="15" customHeight="1">
+      <c r="U24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" ht="15" customHeight="1">
       <c r="A25" s="13" t="s">
         <v>90</v>
       </c>
@@ -2932,7 +2997,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="1:20" ht="15" customHeight="1">
+    <row r="26" spans="1:21" ht="15" customHeight="1">
       <c r="A26" s="13" t="s">
         <v>98</v>
       </c>
@@ -2944,19 +3009,22 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:20" ht="15" customHeight="1">
+    <row r="27" spans="1:21" ht="15" customHeight="1">
       <c r="A27" s="13" t="s">
         <v>99</v>
       </c>
       <c r="B27" s="17">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S27" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="28" spans="1:20" ht="15" customHeight="1">
+      <c r="U27" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" ht="15" customHeight="1">
       <c r="A28" s="13" t="s">
         <v>96</v>
       </c>
@@ -2986,7 +3054,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:20" ht="15" customHeight="1">
+    <row r="29" spans="1:21" ht="15" customHeight="1">
       <c r="A29" s="13" t="s">
         <v>79</v>
       </c>
@@ -3022,7 +3090,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="1:20" ht="15" customHeight="1">
+    <row r="30" spans="1:21" ht="15" customHeight="1">
       <c r="A30" s="13" t="s">
         <v>104</v>
       </c>
@@ -3034,7 +3102,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="1:20" ht="15" customHeight="1">
+    <row r="31" spans="1:21" ht="15" customHeight="1">
       <c r="A31" s="13" t="s">
         <v>105</v>
       </c>
@@ -3049,7 +3117,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="1:20" ht="15" customHeight="1">
+    <row r="32" spans="1:21" ht="15" customHeight="1">
       <c r="A32" s="13" t="s">
         <v>106</v>
       </c>
@@ -3061,7 +3129,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="33" spans="1:20" ht="15" customHeight="1">
+    <row r="33" spans="1:21" ht="15" customHeight="1">
       <c r="A33" s="13" t="s">
         <v>107</v>
       </c>
@@ -3073,7 +3141,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:20" ht="15" customHeight="1">
+    <row r="34" spans="1:21" ht="15" customHeight="1">
       <c r="A34" s="13" t="s">
         <v>108</v>
       </c>
@@ -3085,7 +3153,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:20" ht="15" customHeight="1">
+    <row r="35" spans="1:21" ht="15" customHeight="1">
       <c r="A35" s="13" t="s">
         <v>109</v>
       </c>
@@ -3100,13 +3168,13 @@
         <v>33</v>
       </c>
     </row>
-    <row r="36" spans="1:20" ht="15" customHeight="1">
+    <row r="36" spans="1:21" ht="15" customHeight="1">
       <c r="A36" s="13" t="s">
         <v>110</v>
       </c>
       <c r="B36" s="17">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C36" t="s">
         <v>30</v>
@@ -3153,14 +3221,20 @@
       <c r="T36" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="37" spans="1:20" ht="15" customHeight="1">
+      <c r="U36" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" ht="15" customHeight="1">
       <c r="A37" s="13" t="s">
         <v>112</v>
       </c>
       <c r="B37" s="17">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="U37" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -3168,6 +3242,14 @@
     <mergeCell ref="A1:AA1"/>
   </mergeCells>
   <conditionalFormatting sqref="C4:T36">
+    <cfRule type="cellIs" dxfId="10" priority="6" operator="equal">
+      <formula>"F"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="7" operator="equal">
+      <formula>"P"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:Z29">
     <cfRule type="cellIs" dxfId="8" priority="4" operator="equal">
       <formula>"F"</formula>
     </cfRule>
@@ -3175,16 +3257,16 @@
       <formula>"P"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C4:Z29">
-    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
+  <conditionalFormatting sqref="U36:U37">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"F"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"P"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="C4:Z29 C30:T36" xr:uid="{00000000-0002-0000-0900-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="C4:Z29 C30:T36 U36:U37" xr:uid="{00000000-0002-0000-0900-000000000000}">
       <formula1>"F,P"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3396,23 +3478,23 @@
       </c>
       <c r="B10" s="2">
         <f>COUNTIF('Saisie 2026-06'!Y4:Y30,"Atteint")+COUNTIF('Saisie 2026-06'!Y4:Y30,"Sous objectif")</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" s="2">
         <f>SUM('Saisie 2026-06'!X4:X30)</f>
-        <v>81</v>
+        <v>111</v>
       </c>
       <c r="D10" s="2">
         <f>IFERROR(COUNTIF('Saisie 2026-06'!Y4:Y30,"Atteint")/(COUNTIF('Saisie 2026-06'!Y4:Y30,"Atteint")+COUNTIF('Saisie 2026-06'!Y4:Y30,"Sous objectif")),0)</f>
-        <v>0.61538461538461542</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="E10" s="2">
         <f>IFERROR(SUM('Saisie 2026-06'!X4:X30)/(COUNTIF('Saisie 2026-06'!Y4:Y30,"Atteint")+COUNTIF('Saisie 2026-06'!Y4:Y30,"Sous objectif")),0)</f>
-        <v>3.1153846153846154</v>
+        <v>4.1111111111111107</v>
       </c>
       <c r="F10" s="2">
         <f>COUNTIF('Saisie 2026-06'!X4:X30,"&gt;=1")</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>186</v>
@@ -3424,23 +3506,23 @@
       </c>
       <c r="B11" s="2">
         <f>AVERAGE(B8:B10)</f>
-        <v>26</v>
+        <v>26.333333333333332</v>
       </c>
       <c r="C11" s="2">
         <f>AVERAGE(C8:C10)</f>
-        <v>81.333333333333329</v>
+        <v>91.333333333333329</v>
       </c>
       <c r="D11" s="2">
         <f>AVERAGE(D8:D10)</f>
-        <v>0.66666666666666663</v>
+        <v>0.72079772079772075</v>
       </c>
       <c r="E11" s="2">
         <f>AVERAGE(E8:E10)</f>
-        <v>3.1282051282051282</v>
+        <v>3.4601139601139601</v>
       </c>
       <c r="F11" s="2">
         <f>AVERAGE(F8:F10)</f>
-        <v>24.666666666666668</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -3710,7 +3792,7 @@
       </c>
       <c r="F12" s="2">
         <f>IF('Saisie 2026-06'!Y11="N/A absence longue","M",'Saisie 2026-06'!X11)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G12" s="2">
         <f t="shared" si="0"/>
@@ -3743,15 +3825,15 @@
       </c>
       <c r="F13" s="2">
         <f>IF('Saisie 2026-06'!Y12="N/A absence longue","M",'Saisie 2026-06'!X12)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13" s="2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H13" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>2/5</v>
+        <v>3/5</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15.75" customHeight="1">
@@ -3842,7 +3924,7 @@
       </c>
       <c r="F16" s="2">
         <f>IF('Saisie 2026-06'!Y15="N/A absence longue","M",'Saisie 2026-06'!X15)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G16" s="2">
         <f t="shared" si="0"/>
@@ -3875,7 +3957,7 @@
       </c>
       <c r="F17" s="2">
         <f>IF('Saisie 2026-06'!Y16="N/A absence longue","M",'Saisie 2026-06'!X16)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G17" s="2">
         <f t="shared" si="0"/>
@@ -3908,15 +3990,15 @@
       </c>
       <c r="F18" s="2">
         <f>IF('Saisie 2026-06'!Y17="N/A absence longue","M",'Saisie 2026-06'!X17)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G18" s="2">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H18" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>4/5</v>
+        <v>5/5 ✓</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="15.75" customHeight="1">
@@ -3941,7 +4023,7 @@
       </c>
       <c r="F19" s="2">
         <f>IF('Saisie 2026-06'!Y18="N/A absence longue","M",'Saisie 2026-06'!X18)</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G19" s="2">
         <f t="shared" si="0"/>
@@ -3974,7 +4056,7 @@
       </c>
       <c r="F20" s="2">
         <f>IF('Saisie 2026-06'!Y19="N/A absence longue","M",'Saisie 2026-06'!X19)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G20" s="2">
         <f t="shared" si="0"/>
@@ -4073,7 +4155,7 @@
       </c>
       <c r="F23" s="2">
         <f>IF('Saisie 2026-06'!Y22="N/A absence longue","M",'Saisie 2026-06'!X22)</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G23" s="2">
         <f t="shared" si="0"/>
@@ -4139,15 +4221,15 @@
       </c>
       <c r="F25" s="2">
         <f>IF('Saisie 2026-06'!Y24="N/A absence longue","M",'Saisie 2026-06'!X24)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G25" s="2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H25" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>2/5</v>
+        <v>3/5</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1">
@@ -4271,15 +4353,15 @@
       </c>
       <c r="F29" s="2">
         <f>IF('Saisie 2026-06'!Y28="N/A absence longue","M",'Saisie 2026-06'!X28)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29" s="2">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H29" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>4/5</v>
+        <v>5/5 ✓</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1">
@@ -4304,7 +4386,7 @@
       </c>
       <c r="F30" s="2">
         <f>IF('Saisie 2026-06'!Y29="N/A absence longue","M",'Saisie 2026-06'!X29)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G30" s="2">
         <f t="shared" si="0"/>
@@ -11342,19 +11424,19 @@
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:D1000">
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
       <formula>2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="4" operator="equal">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
       <formula>4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="6" operator="equal">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12882,18 +12964,18 @@
     <mergeCell ref="A1:W1"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:U28">
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="2" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="3" operator="equal">
       <formula>"IC"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="4" operator="equal">
       <formula>"M"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31:U33">
-    <cfRule type="cellIs" dxfId="25" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="5" operator="equal">
       <formula>"X"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14219,18 +14301,18 @@
     <mergeCell ref="A1:Y1"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:W29">
-    <cfRule type="cellIs" dxfId="24" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="2" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="3" operator="equal">
       <formula>"IC"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="4" operator="equal">
       <formula>"M"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32:W34">
-    <cfRule type="cellIs" dxfId="21" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="5" operator="equal">
       <formula>"X"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15532,18 +15614,18 @@
     <mergeCell ref="A1:Y1"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:W29">
-    <cfRule type="cellIs" dxfId="20" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
       <formula>"IC"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="4" operator="equal">
       <formula>"M"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32:W34">
-    <cfRule type="cellIs" dxfId="17" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="5" operator="equal">
       <formula>"X"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16743,18 +16825,18 @@
     <mergeCell ref="A1:U1"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:S29">
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="2" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="3" operator="equal">
       <formula>"IC"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="4" operator="equal">
       <formula>"M"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32:S34">
-    <cfRule type="cellIs" dxfId="13" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="5" operator="equal">
       <formula>"X"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17121,10 +17203,20 @@
         <v>9</v>
       </c>
       <c r="U8" s="14"/>
-      <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
-      <c r="X8" s="17"/>
-      <c r="Y8" s="14"/>
+      <c r="V8" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="W8" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="X8" s="17">
+        <f>COUNTIF(B8:W8,1)+COUNTIF(B8:W8,"IC")</f>
+        <v>17</v>
+      </c>
+      <c r="Y8" s="14" t="str">
+        <f>IF(COUNTIF(B8:W8,"M")&gt;0,"N/A absence longue",IF(X8&gt;=2,"Atteint","Sous objectif"))</f>
+        <v>Atteint</v>
+      </c>
     </row>
     <row r="9" spans="1:25" ht="18" customHeight="1">
       <c r="A9" s="13" t="s">
@@ -17245,10 +17337,12 @@
       </c>
       <c r="U11" s="14"/>
       <c r="V11" s="14"/>
-      <c r="W11" s="14"/>
+      <c r="W11" s="14">
+        <v>1</v>
+      </c>
       <c r="X11" s="17">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y11" s="14" t="str">
         <f t="shared" si="1"/>
@@ -17282,14 +17376,16 @@
       <c r="T12" s="15"/>
       <c r="U12" s="14"/>
       <c r="V12" s="14"/>
-      <c r="W12" s="14"/>
+      <c r="W12" s="14">
+        <v>1</v>
+      </c>
       <c r="X12" s="17">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y12" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>Sous objectif</v>
+        <v>Atteint</v>
       </c>
     </row>
     <row r="13" spans="1:25" ht="18" customHeight="1">
@@ -17399,10 +17495,12 @@
       <c r="T15" s="15"/>
       <c r="U15" s="14"/>
       <c r="V15" s="14"/>
-      <c r="W15" s="14"/>
+      <c r="W15" s="14">
+        <v>1</v>
+      </c>
       <c r="X15" s="17">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y15" s="14" t="str">
         <f t="shared" si="1"/>
@@ -17444,10 +17542,12 @@
       </c>
       <c r="U16" s="14"/>
       <c r="V16" s="14"/>
-      <c r="W16" s="14"/>
+      <c r="W16" s="14">
+        <v>1</v>
+      </c>
       <c r="X16" s="17">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y16" s="14" t="str">
         <f t="shared" si="1"/>
@@ -17481,14 +17581,16 @@
       <c r="T17" s="15"/>
       <c r="U17" s="14"/>
       <c r="V17" s="14"/>
-      <c r="W17" s="14"/>
+      <c r="W17" s="14">
+        <v>1</v>
+      </c>
       <c r="X17" s="17">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y17" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>Sous objectif</v>
+        <v>Atteint</v>
       </c>
     </row>
     <row r="18" spans="1:25" ht="18" customHeight="1">
@@ -17537,11 +17639,15 @@
         <v>9</v>
       </c>
       <c r="U18" s="14"/>
-      <c r="V18" s="14"/>
-      <c r="W18" s="14"/>
+      <c r="V18" s="14">
+        <v>1</v>
+      </c>
+      <c r="W18" s="14" t="s">
+        <v>9</v>
+      </c>
       <c r="X18" s="17">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="Y18" s="14" t="str">
         <f t="shared" si="1"/>
@@ -17577,10 +17683,12 @@
       <c r="T19" s="15"/>
       <c r="U19" s="14"/>
       <c r="V19" s="14"/>
-      <c r="W19" s="14"/>
+      <c r="W19" s="14">
+        <v>1</v>
+      </c>
       <c r="X19" s="17">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y19" s="14" t="str">
         <f t="shared" si="1"/>
@@ -17708,12 +17816,16 @@
       <c r="T22" s="15">
         <v>1</v>
       </c>
-      <c r="U22" s="14"/>
+      <c r="U22" s="14">
+        <v>1</v>
+      </c>
       <c r="V22" s="14"/>
-      <c r="W22" s="14"/>
+      <c r="W22" s="14">
+        <v>1</v>
+      </c>
       <c r="X22" s="17">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Y22" s="14" t="str">
         <f t="shared" si="1"/>
@@ -17783,15 +17895,17 @@
       <c r="S24" s="14"/>
       <c r="T24" s="15"/>
       <c r="U24" s="14"/>
-      <c r="V24" s="14"/>
+      <c r="V24" s="14">
+        <v>1</v>
+      </c>
       <c r="W24" s="14"/>
       <c r="X24" s="17">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y24" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>Sous objectif</v>
+        <v>Atteint</v>
       </c>
     </row>
     <row r="25" spans="1:25" ht="18" customHeight="1">
@@ -17928,14 +18042,16 @@
       <c r="T28" s="15"/>
       <c r="U28" s="14"/>
       <c r="V28" s="14"/>
-      <c r="W28" s="14"/>
+      <c r="W28" s="14">
+        <v>1</v>
+      </c>
       <c r="X28" s="17">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y28" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>Sous objectif</v>
+        <v>Atteint</v>
       </c>
     </row>
     <row r="29" spans="1:25" ht="18" customHeight="1">
@@ -17967,10 +18083,12 @@
       <c r="T29" s="15"/>
       <c r="U29" s="14"/>
       <c r="V29" s="14"/>
-      <c r="W29" s="14"/>
+      <c r="W29" s="14">
+        <v>1</v>
+      </c>
       <c r="X29" s="17">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y29" s="14" t="str">
         <f t="shared" si="1"/>
@@ -18117,18 +18235,18 @@
     <mergeCell ref="A1:Y1"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:W30">
-    <cfRule type="cellIs" dxfId="12" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="2" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="3" operator="equal">
       <formula>"IC"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="4" operator="equal">
       <formula>"M"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33:W35">
-    <cfRule type="cellIs" dxfId="9" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="5" operator="equal">
       <formula>"X"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18438,7 +18556,18 @@
       </c>
     </row>
     <row r="22" spans="1:4" ht="15" customHeight="1">
-      <c r="B22" s="7"/>
+      <c r="A22" t="s">
+        <v>393</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>394</v>
+      </c>
+      <c r="C22" t="s">
+        <v>395</v>
+      </c>
+      <c r="D22" t="s">
+        <v>396</v>
+      </c>
     </row>
     <row r="23" spans="1:4" ht="15" customHeight="1">
       <c r="B23" s="7"/>
@@ -18675,6 +18804,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
+  <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix date F-2026-010 (texte -> date Excel)
</commit_message>
<xml_diff>
--- a/public/data/suivi_presence_consultants.xlsx
+++ b/public/data/suivi_presence_consultants.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeremiekieffer/Projets/ikxo-presence-dashboard/public/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E89EBFD8-7396-4D4D-B94C-F02542D0E4C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B670180-3E41-E54A-9ED9-DE64F0CBFE13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17520" tabRatio="500" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17520" tabRatio="500" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Convention" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1101" uniqueCount="396">
   <si>
     <t>Convention de saisie — Suivi de présence consultants</t>
   </si>
@@ -1275,9 +1275,6 @@
   </si>
   <si>
     <t>F-2026-010</t>
-  </si>
-  <si>
-    <t>06/30/2026</t>
   </si>
   <si>
     <t>Tech For PM#3 - Data Model</t>
@@ -18559,14 +18556,14 @@
       <c r="A22" t="s">
         <v>393</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="7">
+        <v>46203</v>
+      </c>
+      <c r="C22" t="s">
         <v>394</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>395</v>
-      </c>
-      <c r="D22" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="15" customHeight="1">

</xml_diff>